<commit_message>
fix: standardize date format to YYYY-MM-DD and publish registry entry (#39)
Convert lending rate dates from YYYY-MM to YYYY-MM-01 to match project
convention. Also run registry publish to assign permanent URL.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data.mn/public/datasets/mongolbank-lending-rate-mnt-monthly.xlsx
+++ b/data.mn/public/datasets/mongolbank-lending-rate-mnt-monthly.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2016-03</t>
+          <t>2016-03-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -442,7 +442,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2016-04</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -452,7 +452,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2016-05</t>
+          <t>2016-05-01</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -462,7 +462,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2016-06</t>
+          <t>2016-06-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -472,7 +472,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2016-07</t>
+          <t>2016-07-01</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -482,7 +482,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2016-08</t>
+          <t>2016-08-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -492,7 +492,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2016-09</t>
+          <t>2016-09-01</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -502,7 +502,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2016-10</t>
+          <t>2016-10-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -512,7 +512,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2016-11</t>
+          <t>2016-11-01</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -522,7 +522,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2016-12</t>
+          <t>2016-12-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -532,7 +532,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2017-01</t>
+          <t>2017-01-01</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -542,7 +542,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2017-02</t>
+          <t>2017-02-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -552,7 +552,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2017-03</t>
+          <t>2017-03-01</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -562,7 +562,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2017-04</t>
+          <t>2017-04-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -572,7 +572,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2017-05</t>
+          <t>2017-05-01</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -582,7 +582,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2017-06</t>
+          <t>2017-06-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -592,7 +592,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2017-07</t>
+          <t>2017-07-01</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -602,7 +602,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2017-08</t>
+          <t>2017-08-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -612,7 +612,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2017-09</t>
+          <t>2017-09-01</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -622,7 +622,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2017-10</t>
+          <t>2017-10-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -632,7 +632,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2017-11</t>
+          <t>2017-11-01</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -642,7 +642,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2017-12</t>
+          <t>2017-12-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -652,7 +652,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2018-01</t>
+          <t>2018-01-01</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -662,7 +662,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2018-02</t>
+          <t>2018-02-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -672,7 +672,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2018-03</t>
+          <t>2018-03-01</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -682,7 +682,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2018-04</t>
+          <t>2018-04-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -692,7 +692,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2018-05</t>
+          <t>2018-05-01</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -702,7 +702,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2018-06</t>
+          <t>2018-06-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -712,7 +712,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2018-07</t>
+          <t>2018-07-01</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -722,7 +722,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2018-08</t>
+          <t>2018-08-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -732,7 +732,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2018-09</t>
+          <t>2018-09-01</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -742,7 +742,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2018-10</t>
+          <t>2018-10-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -752,7 +752,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2018-11</t>
+          <t>2018-11-01</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -762,7 +762,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2018-12</t>
+          <t>2018-12-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -772,7 +772,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2019-01</t>
+          <t>2019-01-01</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -782,7 +782,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2019-02</t>
+          <t>2019-02-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -792,7 +792,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2019-03</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -802,7 +802,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2019-04</t>
+          <t>2019-04-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -812,7 +812,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2019-05</t>
+          <t>2019-05-01</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -822,7 +822,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2019-06</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -832,7 +832,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2019-07</t>
+          <t>2019-07-01</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -842,7 +842,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2019-08</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -852,7 +852,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2019-09</t>
+          <t>2019-09-01</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -862,7 +862,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2019-10</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -872,7 +872,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2019-11</t>
+          <t>2019-11-01</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -882,7 +882,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2019-12</t>
+          <t>2019-12-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -892,7 +892,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2020-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -902,7 +902,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2020-02</t>
+          <t>2020-02-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -912,7 +912,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2020-03</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -922,7 +922,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2020-04</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -932,7 +932,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2020-05</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -942,7 +942,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2020-06</t>
+          <t>2020-06-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -952,7 +952,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2020-07</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -962,7 +962,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2020-08</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -972,7 +972,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2020-09</t>
+          <t>2020-09-01</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -982,7 +982,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2020-10</t>
+          <t>2020-10-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -992,7 +992,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2020-11</t>
+          <t>2020-11-01</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1002,7 +1002,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2020-12</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1012,7 +1012,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2021-01</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1022,7 +1022,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2021-02</t>
+          <t>2021-02-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1032,7 +1032,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2021-03</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1042,7 +1042,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2021-04</t>
+          <t>2021-04-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1052,7 +1052,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2021-05</t>
+          <t>2021-05-01</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1062,7 +1062,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2021-06</t>
+          <t>2021-06-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1072,7 +1072,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2021-07</t>
+          <t>2021-07-01</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1082,7 +1082,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2021-08</t>
+          <t>2021-08-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1092,7 +1092,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2021-09</t>
+          <t>2021-09-01</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1102,7 +1102,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2021-10</t>
+          <t>2021-10-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1112,7 +1112,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2021-11-01</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1122,7 +1122,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2021-12</t>
+          <t>2021-12-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1132,7 +1132,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2022-01</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1142,7 +1142,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2022-02</t>
+          <t>2022-02-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1152,7 +1152,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2022-03</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1162,7 +1162,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2022-04</t>
+          <t>2022-04-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1172,7 +1172,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2022-05</t>
+          <t>2022-05-01</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1182,7 +1182,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2022-06</t>
+          <t>2022-06-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1192,7 +1192,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2022-07</t>
+          <t>2022-07-01</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1202,7 +1202,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2022-08</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1212,7 +1212,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2022-09</t>
+          <t>2022-09-01</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1222,7 +1222,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2022-10</t>
+          <t>2022-10-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1232,7 +1232,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2022-11</t>
+          <t>2022-11-01</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1242,7 +1242,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2022-12</t>
+          <t>2022-12-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1252,7 +1252,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2023-01-01</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1262,7 +1262,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2023-02-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1272,7 +1272,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2023-03</t>
+          <t>2023-03-01</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1282,7 +1282,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2023-04</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1292,7 +1292,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2023-05-01</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1302,7 +1302,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2023-06-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1312,7 +1312,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2023-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1322,7 +1322,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1332,7 +1332,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2023-09-01</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1342,7 +1342,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-10-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1352,7 +1352,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-11-01</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1362,7 +1362,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2023-12-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1372,7 +1372,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1382,7 +1382,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1392,7 +1392,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1402,7 +1402,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-04-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1412,7 +1412,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-05-01</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1422,7 +1422,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1432,7 +1432,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1442,7 +1442,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -1452,7 +1452,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-09-01</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1462,7 +1462,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -1472,7 +1472,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -1482,7 +1482,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -1492,7 +1492,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -1502,7 +1502,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -1512,7 +1512,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-03-01</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -1522,7 +1522,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-04-01</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -1532,7 +1532,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -1542,7 +1542,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-06-01</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -1552,7 +1552,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -1562,7 +1562,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1572,7 +1572,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1582,7 +1582,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -1592,7 +1592,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1602,7 +1602,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1612,7 +1612,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -1648,7 +1648,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2016-03</t>
+          <t>2016-03-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1658,7 +1658,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2016-04</t>
+          <t>2016-04-01</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1668,7 +1668,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2016-05</t>
+          <t>2016-05-01</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1678,7 +1678,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2016-06</t>
+          <t>2016-06-01</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1688,7 +1688,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2016-07</t>
+          <t>2016-07-01</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1698,7 +1698,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2016-08</t>
+          <t>2016-08-01</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1708,7 +1708,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2016-09</t>
+          <t>2016-09-01</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1718,7 +1718,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2016-10</t>
+          <t>2016-10-01</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1728,7 +1728,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2016-11</t>
+          <t>2016-11-01</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1738,7 +1738,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2016-12</t>
+          <t>2016-12-01</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1748,7 +1748,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2017-01</t>
+          <t>2017-01-01</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1758,7 +1758,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2017-02</t>
+          <t>2017-02-01</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1768,7 +1768,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2017-03</t>
+          <t>2017-03-01</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1778,7 +1778,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2017-04</t>
+          <t>2017-04-01</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1788,7 +1788,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2017-05</t>
+          <t>2017-05-01</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1798,7 +1798,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2017-06</t>
+          <t>2017-06-01</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1808,7 +1808,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2017-07</t>
+          <t>2017-07-01</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1818,7 +1818,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2017-08</t>
+          <t>2017-08-01</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1828,7 +1828,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2017-09</t>
+          <t>2017-09-01</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1838,7 +1838,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2017-10</t>
+          <t>2017-10-01</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1848,7 +1848,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2017-11</t>
+          <t>2017-11-01</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1858,7 +1858,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2017-12</t>
+          <t>2017-12-01</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1868,7 +1868,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2018-01</t>
+          <t>2018-01-01</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1878,7 +1878,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2018-02</t>
+          <t>2018-02-01</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1888,7 +1888,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2018-03</t>
+          <t>2018-03-01</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1898,7 +1898,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2018-04</t>
+          <t>2018-04-01</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1908,7 +1908,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2018-05</t>
+          <t>2018-05-01</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1918,7 +1918,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2018-06</t>
+          <t>2018-06-01</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1928,7 +1928,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2018-07</t>
+          <t>2018-07-01</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1938,7 +1938,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2018-08</t>
+          <t>2018-08-01</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1948,7 +1948,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2018-09</t>
+          <t>2018-09-01</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1958,7 +1958,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2018-10</t>
+          <t>2018-10-01</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1968,7 +1968,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2018-11</t>
+          <t>2018-11-01</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1978,7 +1978,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2018-12</t>
+          <t>2018-12-01</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1988,7 +1988,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2019-01</t>
+          <t>2019-01-01</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1998,7 +1998,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2019-02</t>
+          <t>2019-02-01</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2008,7 +2008,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2019-03</t>
+          <t>2019-03-01</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2018,7 +2018,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2019-04</t>
+          <t>2019-04-01</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2028,7 +2028,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2019-05</t>
+          <t>2019-05-01</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2038,7 +2038,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2019-06</t>
+          <t>2019-06-01</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2048,7 +2048,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2019-07</t>
+          <t>2019-07-01</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -2058,7 +2058,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2019-08</t>
+          <t>2019-08-01</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -2068,7 +2068,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2019-09</t>
+          <t>2019-09-01</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -2078,7 +2078,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2019-10</t>
+          <t>2019-10-01</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -2088,7 +2088,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2019-11</t>
+          <t>2019-11-01</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -2098,7 +2098,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2019-12</t>
+          <t>2019-12-01</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -2108,7 +2108,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2020-01</t>
+          <t>2020-01-01</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -2118,7 +2118,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2020-02</t>
+          <t>2020-02-01</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -2128,7 +2128,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2020-03</t>
+          <t>2020-03-01</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -2138,7 +2138,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2020-04</t>
+          <t>2020-04-01</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -2148,7 +2148,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2020-05</t>
+          <t>2020-05-01</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -2158,7 +2158,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2020-06</t>
+          <t>2020-06-01</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -2168,7 +2168,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2020-07</t>
+          <t>2020-07-01</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -2178,7 +2178,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2020-08</t>
+          <t>2020-08-01</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -2188,7 +2188,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2020-09</t>
+          <t>2020-09-01</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -2198,7 +2198,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2020-10</t>
+          <t>2020-10-01</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -2208,7 +2208,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2020-11</t>
+          <t>2020-11-01</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -2218,7 +2218,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2020-12</t>
+          <t>2020-12-01</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -2228,7 +2228,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2021-01</t>
+          <t>2021-01-01</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -2238,7 +2238,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2021-02</t>
+          <t>2021-02-01</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2248,7 +2248,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2021-03</t>
+          <t>2021-03-01</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -2258,7 +2258,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2021-04</t>
+          <t>2021-04-01</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -2268,7 +2268,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2021-05</t>
+          <t>2021-05-01</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -2278,7 +2278,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2021-06</t>
+          <t>2021-06-01</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -2288,7 +2288,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2021-07</t>
+          <t>2021-07-01</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -2298,7 +2298,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2021-08</t>
+          <t>2021-08-01</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -2308,7 +2308,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2021-09</t>
+          <t>2021-09-01</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -2318,7 +2318,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2021-10</t>
+          <t>2021-10-01</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -2328,7 +2328,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2021-11</t>
+          <t>2021-11-01</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -2338,7 +2338,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2021-12</t>
+          <t>2021-12-01</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -2348,7 +2348,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2022-01</t>
+          <t>2022-01-01</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -2358,7 +2358,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2022-02</t>
+          <t>2022-02-01</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2368,7 +2368,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2022-03</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -2378,7 +2378,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2022-04</t>
+          <t>2022-04-01</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -2388,7 +2388,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2022-05</t>
+          <t>2022-05-01</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -2398,7 +2398,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2022-06</t>
+          <t>2022-06-01</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -2408,7 +2408,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2022-07</t>
+          <t>2022-07-01</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -2418,7 +2418,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2022-08</t>
+          <t>2022-08-01</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -2428,7 +2428,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2022-09</t>
+          <t>2022-09-01</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -2438,7 +2438,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2022-10</t>
+          <t>2022-10-01</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -2448,7 +2448,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2022-11</t>
+          <t>2022-11-01</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2458,7 +2458,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2022-12</t>
+          <t>2022-12-01</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -2468,7 +2468,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2023-01-01</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -2478,7 +2478,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2023-02-01</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2488,7 +2488,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2023-03</t>
+          <t>2023-03-01</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2023-04</t>
+          <t>2023-04-01</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2508,7 +2508,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2023-05-01</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2518,7 +2518,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2023-06-01</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -2528,7 +2528,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2023-07</t>
+          <t>2023-07-01</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2538,7 +2538,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2023-08-01</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2548,7 +2548,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2023-09-01</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -2558,7 +2558,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-10-01</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2568,7 +2568,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-11-01</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2578,7 +2578,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2023-12-01</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2588,7 +2588,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-01-01</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2598,7 +2598,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-02-01</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2608,7 +2608,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-03-01</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2618,7 +2618,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-04-01</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2628,7 +2628,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-05-01</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2638,7 +2638,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-06-01</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2648,7 +2648,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-07-01</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2658,7 +2658,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-08-01</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2668,7 +2668,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-09-01</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2678,7 +2678,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2688,7 +2688,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2698,7 +2698,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-12-01</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2708,7 +2708,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-01-01</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2718,7 +2718,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-02-01</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2728,7 +2728,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-03-01</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2738,7 +2738,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-04-01</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2748,7 +2748,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-05-01</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -2758,7 +2758,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-06-01</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -2768,7 +2768,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-07-01</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -2778,7 +2778,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2025-08-01</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2788,7 +2788,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2025-09-01</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2798,7 +2798,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2025-10-01</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -2808,7 +2808,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2025-11-01</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2818,7 +2818,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2025-12-01</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2828,7 +2828,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-01-01</t>
         </is>
       </c>
       <c r="B120" t="n">

</xml_diff>